<commit_message>
Add import templates for customers and contacts
Customers come first in the import order: the customer_code filled in
there is what the contact, site and contract templates match on. Contacts
follow, linking back by that same code.

Both are optional columns as far as the schema goes, so they get a third
header colour — amber for "blank is legal but breaks the chain" — sitting
between the required orange and the optional green. The existing three
templates use it for their customer_code too.

Phone and tax-id columns are formatted as text so leading zeros survive.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/import-templates/import-template-assets.xlsx
+++ b/import-templates/import-template-assets.xlsx
@@ -50,7 +50,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -72,6 +72,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF3F4F6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFB45309"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -103,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -127,6 +133,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -638,7 +647,7 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">หัวคอลัมน์สีส้ม = จำเป็นต้องกรอก / สีเขียว = ไม่บังคับ (เว้นว่างได้)</t>
+          <t xml:space="preserve">หัวคอลัมน์สีส้ม = จำเป็นต้องกรอก / สีเหลือง = ไม่บังคับ แต่แนะนำอย่างยิ่ง / สีเขียว = เว้นว่างได้</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Match customers by tax id, not customer code
Checked the live data before these templates get filled in: of 31
customers, only 4 carry a customer_code but 26 carry a tax_id. Keying the
contact, site and contract templates on customer_code would therefore
have failed to match most existing customers.

So tax_id becomes the amber "fill this in" column and customer_code
demotes to green, with every lookup running customer_code -> tax_id ->
company_name. Worked examples now follow the conventions the real rows
use: observed customer_code shapes, the tag vocabulary actually in use,
coordinates in the address field, and technician names as spelled.

checkSpec() guards the example rows against drifting out of step with the
columns — it caught the contract examples missing company_name.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/import-templates/import-template-assets.xlsx
+++ b/import-templates/import-template-assets.xlsx
@@ -349,7 +349,7 @@
     <row r="2">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">โรงงานบางปู เฟส 2</t>
+          <t xml:space="preserve">PT บางปู สมุทรปราการ</t>
         </is>
       </c>
       <c r="B2" s="9" t="inlineStr">
@@ -413,12 +413,12 @@
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">โรงงานบางปู เฟส 2</t>
+          <t xml:space="preserve">PT บางปู สมุทรปราการ</t>
         </is>
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">แผงโซลาร์ ชุดหลังคา A</t>
+          <t xml:space="preserve">ตู้เติมลมโครงเหล็ก-Outdoor</t>
         </is>
       </c>
       <c r="C3" s="9" t="inlineStr">
@@ -428,22 +428,18 @@
       </c>
       <c r="D3" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">solar_panel</t>
+          <t xml:space="preserve">other</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jinko</t>
-        </is>
-      </c>
-      <c r="F3" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">JKM580N-72HL4</t>
-        </is>
-      </c>
+          <t xml:space="preserve">G5</t>
+        </is>
+      </c>
+      <c r="F3" s="9"/>
       <c r="G3" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">JK24A0099123</t>
+          <t xml:space="preserve">6972220250521</t>
         </is>
       </c>
       <c r="H3" s="9"/>
@@ -464,7 +460,7 @@
       </c>
       <c r="L3" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">144</t>
+          <t xml:space="preserve">24</t>
         </is>
       </c>
       <c r="M3" s="9" t="inlineStr">
@@ -474,7 +470,7 @@
       </c>
       <c r="N3" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">รวม 320 แผง</t>
+          <t xml:space="preserve">ประเภทที่ไม่เข้าพวกให้ใช้ other</t>
         </is>
       </c>
     </row>
@@ -530,14 +526,14 @@
       </c>
       <c r="N4" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">โครงการเฟสแรก</t>
+          <t xml:space="preserve">asset_type = project จึงกรอก project_number แทน serial_number</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">สาขาระยอง (หลังคาอาคาร A)</t>
+          <t xml:space="preserve">สาขาระยอง (อาคาร A)</t>
         </is>
       </c>
       <c r="B5" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Narrow the site list to the sites holding a given machine
A branch that has a Probe due for calibration is not something the site
list could answer: it knew only how many machines a site held, not what
they were.

Each site now carries the kinds, brands and models it holds, and the
toolbar offers one type-to-search filter per facet, each option showing
how many sites it would leave. The kinds are also written under the
count, so a site that survives a filter says why.

The values are aggregated by a view rather than by fetching all 5,877
equipment rows per page load, and reach the browser as indices into one
shared vocabulary — the model names alone repeat to 276 KB when sent as
strings, against 84 KB as numbers.

The assets template picked up the company_name column it was already
being generated with.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/import-templates/import-template-assets.xlsx
+++ b/import-templates/import-template-assets.xlsx
@@ -146,24 +146,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:P1"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="13" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="20" customWidth="1"/>
-    <col min="8" max="8" width="22" customWidth="1"/>
-    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="3" max="3" width="30" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="13" customWidth="1"/>
+    <col min="6" max="6" width="26" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="8" max="8" width="20" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
     <col min="10" max="10" width="18" customWidth="1"/>
-    <col min="11" max="11" width="15" customWidth="1" style="3"/>
-    <col min="12" max="12" width="16" customWidth="1" style="3"/>
-    <col min="13" max="13" width="15" customWidth="1"/>
-    <col min="14" max="14" width="14" customWidth="1"/>
-    <col min="15" max="15" width="30" customWidth="1"/>
+    <col min="11" max="11" width="18" customWidth="1"/>
+    <col min="12" max="12" width="15" customWidth="1" style="3"/>
+    <col min="13" max="13" width="16" customWidth="1" style="3"/>
+    <col min="14" max="14" width="15" customWidth="1"/>
+    <col min="15" max="15" width="14" customWidth="1"/>
+    <col min="16" max="16" width="30" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -172,87 +173,89 @@
           <t xml:space="preserve">site_name</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">company_name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">asset_tag</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">asset_type</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">category</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">brand</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">model</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">serial_number</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">project_number</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">group_name</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">install_date</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">warranty_start</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">warranty_months</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">status</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">notes</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O1"/>
-  <dataValidations count="3">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="ค่าไม่ถูกต้อง" error="กรุณาเลือกจากรายการที่กำหนด" sqref="D2:D2000">
+  <autoFilter ref="A1:P1"/>
+  <dataValidations count="2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="ค่าไม่ถูกต้อง" error="กรุณาเลือกจากรายการที่กำหนด" sqref="E2:E2000">
       <formula1>"object,project"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="ค่าไม่ถูกต้อง" error="กรุณาเลือกจากรายการที่กำหนด" sqref="E2:E2000">
-      <formula1>"solar_panel,inverter,ev_charger,battery,meter,other"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="ค่าไม่ถูกต้อง" error="กรุณาเลือกจากรายการที่กำหนด" sqref="N2:N2000">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="ค่าไม่ถูกต้อง" error="กรุณาเลือกจากรายการที่กำหนด" sqref="O2:O2000">
       <formula1>"operational,degraded,down,retired"</formula1>
     </dataValidation>
   </dataValidations>
@@ -261,24 +264,25 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:O7"/>
+  <dimension ref="A1:P7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
-    <col min="4" max="4" width="13" customWidth="1"/>
-    <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="16" customWidth="1"/>
-    <col min="7" max="7" width="20" customWidth="1"/>
-    <col min="8" max="8" width="22" customWidth="1"/>
-    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="3" max="3" width="30" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="13" customWidth="1"/>
+    <col min="6" max="6" width="26" customWidth="1"/>
+    <col min="7" max="7" width="16" customWidth="1"/>
+    <col min="8" max="8" width="20" customWidth="1"/>
+    <col min="9" max="9" width="22" customWidth="1"/>
     <col min="10" max="10" width="18" customWidth="1"/>
-    <col min="11" max="11" width="15" customWidth="1"/>
-    <col min="12" max="12" width="16" customWidth="1"/>
-    <col min="13" max="13" width="15" customWidth="1"/>
-    <col min="14" max="14" width="14" customWidth="1"/>
-    <col min="15" max="15" width="30" customWidth="1"/>
+    <col min="11" max="11" width="18" customWidth="1"/>
+    <col min="12" max="12" width="15" customWidth="1"/>
+    <col min="13" max="13" width="16" customWidth="1"/>
+    <col min="14" max="14" width="15" customWidth="1"/>
+    <col min="15" max="15" width="14" customWidth="1"/>
+    <col min="16" max="16" width="30" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -287,72 +291,77 @@
           <t xml:space="preserve">site_name</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">company_name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">asset_tag</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">asset_type</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">category</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">brand</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">model</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">serial_number</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">project_number</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">group_name</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">install_date</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">warranty_start</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">warranty_months</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">status</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">notes</t>
         </is>
@@ -366,66 +375,71 @@
       </c>
       <c r="B2" s="9" t="inlineStr">
         <is>
+          <t xml:space="preserve">บริษัท ไทยรุ่งเรือง ปิโตรเลียม จำกัด</t>
+        </is>
+      </c>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
           <t xml:space="preserve">อินเวอร์เตอร์ตัวที่ 1</t>
         </is>
       </c>
-      <c r="C2" s="9" t="inlineStr">
+      <c r="D2" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">INV-001</t>
         </is>
       </c>
-      <c r="D2" s="9" t="inlineStr">
+      <c r="E2" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">object</t>
         </is>
       </c>
-      <c r="E2" s="9" t="inlineStr">
+      <c r="F2" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">inverter</t>
         </is>
       </c>
-      <c r="F2" s="9" t="inlineStr">
+      <c r="G2" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Huawei</t>
         </is>
       </c>
-      <c r="G2" s="9" t="inlineStr">
+      <c r="H2" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">SUN2000-100KTL-M1</t>
         </is>
       </c>
-      <c r="H2" s="9" t="inlineStr">
+      <c r="I2" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">HV2340019876</t>
         </is>
       </c>
-      <c r="I2" s="9"/>
-      <c r="J2" s="9" t="inlineStr">
+      <c r="J2" s="9"/>
+      <c r="K2" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">อาคาร A</t>
         </is>
       </c>
-      <c r="K2" s="9" t="inlineStr">
+      <c r="L2" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">2024-06-12</t>
         </is>
       </c>
-      <c r="L2" s="9" t="inlineStr">
+      <c r="M2" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">2024-06-12</t>
         </is>
       </c>
-      <c r="M2" s="9" t="inlineStr">
+      <c r="N2" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">60</t>
         </is>
       </c>
-      <c r="N2" s="9" t="inlineStr">
+      <c r="O2" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">operational</t>
         </is>
       </c>
-      <c r="O2" s="9"/>
+      <c r="P2" s="9"/>
     </row>
     <row r="3">
       <c r="A3" s="9" t="inlineStr">
@@ -435,62 +449,67 @@
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
+          <t xml:space="preserve">บริษัท ไทยรุ่งเรือง ปิโตรเลียม จำกัด</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
           <t xml:space="preserve">ตู้เติมลมโครงเหล็ก-Outdoor</t>
         </is>
       </c>
-      <c r="C3" s="9" t="inlineStr">
+      <c r="D3" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">AIR-014</t>
         </is>
       </c>
-      <c r="D3" s="9" t="inlineStr">
+      <c r="E3" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">object</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr">
+      <c r="F3" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">other</t>
         </is>
       </c>
-      <c r="F3" s="9" t="inlineStr">
+      <c r="G3" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">G5</t>
         </is>
       </c>
-      <c r="G3" s="9"/>
-      <c r="H3" s="9" t="inlineStr">
+      <c r="H3" s="9"/>
+      <c r="I3" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">6972220250521</t>
         </is>
       </c>
-      <c r="I3" s="9"/>
-      <c r="J3" s="9" t="inlineStr">
+      <c r="J3" s="9"/>
+      <c r="K3" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">อาคาร A</t>
         </is>
       </c>
-      <c r="K3" s="9" t="inlineStr">
+      <c r="L3" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">2024-06-12</t>
         </is>
       </c>
-      <c r="L3" s="9" t="inlineStr">
+      <c r="M3" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">2024-06-12</t>
         </is>
       </c>
-      <c r="M3" s="9" t="inlineStr">
+      <c r="N3" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">24</t>
         </is>
       </c>
-      <c r="N3" s="9" t="inlineStr">
+      <c r="O3" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">operational</t>
         </is>
       </c>
-      <c r="O3" s="9" t="inlineStr">
+      <c r="P3" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">ประเภทที่ไม่เข้าพวกให้ใช้ other</t>
         </is>
@@ -504,50 +523,55 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
+          <t xml:space="preserve">ห้างหุ้นส่วนจำกัด เอ็นเนอร์ยี่ พลัส</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
           <t xml:space="preserve">โครงการติดตั้งโซลาร์ 1.2 MW</t>
         </is>
       </c>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9" t="inlineStr">
+      <c r="D4" s="9"/>
+      <c r="E4" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">project</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr">
+      <c r="F4" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">other</t>
         </is>
       </c>
-      <c r="F4" s="9"/>
       <c r="G4" s="9"/>
       <c r="H4" s="9"/>
-      <c r="I4" s="9" t="inlineStr">
+      <c r="I4" s="9"/>
+      <c r="J4" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">PRJ-2024-0087</t>
         </is>
       </c>
-      <c r="J4" s="9"/>
-      <c r="K4" s="9" t="inlineStr">
+      <c r="K4" s="9"/>
+      <c r="L4" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">2024-11-01</t>
         </is>
       </c>
-      <c r="L4" s="9" t="inlineStr">
+      <c r="M4" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">2024-11-01</t>
         </is>
       </c>
-      <c r="M4" s="9" t="inlineStr">
+      <c r="N4" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">60</t>
         </is>
       </c>
-      <c r="N4" s="9" t="inlineStr">
+      <c r="O4" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">operational</t>
         </is>
       </c>
-      <c r="O4" s="9" t="inlineStr">
+      <c r="P4" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">asset_type = project จึงกรอก project_number แทน serial_number</t>
         </is>
@@ -561,62 +585,67 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
+          <t xml:space="preserve">บริษัท สุขสบาย เซอร์วิส จำกัด</t>
+        </is>
+      </c>
+      <c r="C5" s="9" t="inlineStr">
+        <is>
           <t xml:space="preserve">ตู้ชาร์จ EV จุดที่ 3</t>
         </is>
       </c>
-      <c r="C5" s="9" t="inlineStr">
+      <c r="D5" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">EV-003</t>
         </is>
       </c>
-      <c r="D5" s="9" t="inlineStr">
+      <c r="E5" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">object</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">ev_charger</t>
         </is>
       </c>
-      <c r="F5" s="9" t="inlineStr">
+      <c r="G5" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">Delta</t>
         </is>
       </c>
-      <c r="G5" s="9" t="inlineStr">
+      <c r="H5" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">AC Max 22kW</t>
         </is>
       </c>
-      <c r="H5" s="9" t="inlineStr">
+      <c r="I5" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">DL2412000455</t>
         </is>
       </c>
-      <c r="I5" s="9"/>
       <c r="J5" s="9"/>
-      <c r="K5" s="9" t="inlineStr">
+      <c r="K5" s="9"/>
+      <c r="L5" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">2025-02-20</t>
         </is>
       </c>
-      <c r="L5" s="9" t="inlineStr">
+      <c r="M5" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">2025-02-20</t>
         </is>
       </c>
-      <c r="M5" s="9" t="inlineStr">
+      <c r="N5" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">24</t>
         </is>
       </c>
-      <c r="N5" s="9" t="inlineStr">
+      <c r="O5" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">degraded</t>
         </is>
       </c>
-      <c r="O5" s="9" t="inlineStr">
+      <c r="P5" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">จอแสดงผลมีปัญหา รอเปลี่ยนอะไหล่</t>
         </is>
@@ -636,7 +665,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -766,12 +795,12 @@
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">name</t>
+          <t xml:space="preserve">company_name</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ใช่</t>
+          <t xml:space="preserve">—</t>
         </is>
       </c>
       <c r="D13" s="8" t="inlineStr">
@@ -781,7 +810,7 @@
       </c>
       <c r="E13" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">ชื่อ Asset เช่น “อินเวอร์เตอร์ตัวที่ 1” หรือชื่อโครงการ</t>
+          <t xml:space="preserve">ชื่อลูกค้าเจ้าของไซต์ — จำเป็นเมื่อมีไซต์ชื่อซ้ำกันหลายราย (เช่น “ระยอง” มี 9 แห่งคนละลูกค้า) ถ้าชื่อไซต์ไม่ซ้ำจะเว้นว่างได้</t>
         </is>
       </c>
     </row>
@@ -793,12 +822,12 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">asset_tag</t>
+          <t xml:space="preserve">name</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">—</t>
+          <t xml:space="preserve">ใช่</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
@@ -808,7 +837,7 @@
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">เลขครุภัณฑ์ / QR Code ที่ติดอยู่บนเครื่อง เช่น Shell-001 — คนละอันกับรหัส Asset (AS-0001) ที่ระบบออกให้เอง</t>
+          <t xml:space="preserve">ชื่อ Asset เช่น “อินเวอร์เตอร์ตัวที่ 1” หรือชื่อโครงการ</t>
         </is>
       </c>
     </row>
@@ -820,22 +849,22 @@
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">asset_type</t>
+          <t xml:space="preserve">asset_tag</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">ใช่</t>
+          <t xml:space="preserve">—</t>
         </is>
       </c>
       <c r="D15" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">ตัวเลือก: object / project</t>
+          <t xml:space="preserve">ข้อความ</t>
         </is>
       </c>
       <c r="E15" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">object = อุปกรณ์ชิ้นจริง ระบุด้วย serial_number · project = โครงการ ระบุด้วย project_number</t>
+          <t xml:space="preserve">เลขครุภัณฑ์ / QR Code ที่ติดอยู่บนเครื่อง เช่น Shell-001 — คนละอันกับรหัส Asset (AS-0001) ที่ระบบออกให้เอง</t>
         </is>
       </c>
     </row>
@@ -847,7 +876,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">category</t>
+          <t xml:space="preserve">asset_type</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -857,12 +886,12 @@
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">ตัวเลือก: solar_panel / inverter / ev_charger / battery / meter / other</t>
+          <t xml:space="preserve">ตัวเลือก: object / project</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">ประเภท: solar_panel = แผงโซลาร์, inverter = อินเวอร์เตอร์, ev_charger = ตู้ชาร์จ EV, battery = แบตเตอรี่, meter = มิเตอร์, other = อื่นๆ</t>
+          <t xml:space="preserve">object = อุปกรณ์ชิ้นจริง ระบุด้วย serial_number · project = โครงการ ระบุด้วย project_number</t>
         </is>
       </c>
     </row>
@@ -874,12 +903,12 @@
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">brand</t>
+          <t xml:space="preserve">category</t>
         </is>
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">—</t>
+          <t xml:space="preserve">ใช่</t>
         </is>
       </c>
       <c r="D17" s="8" t="inlineStr">
@@ -889,7 +918,7 @@
       </c>
       <c r="E17" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">ยี่ห้อ เช่น Huawei, Growatt, Delta</t>
+          <t xml:space="preserve">ชนิดเครื่อง เช่น “Probe”, “Liquid Sensor”, “Nozzle (หัวฉีด)” — พิมพ์ได้อิสระ ไม่จำกัดตัวเลือก · ค่าที่ระบบมีคำแปลไทยให้: solar_panel = แผงโซลาร์, inverter = อินเวอร์เตอร์, ev_charger = ตู้ชาร์จ EV, battery = แบตเตอรี่, meter = มิเตอร์, other = อื่นๆ</t>
         </is>
       </c>
     </row>
@@ -901,7 +930,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">model</t>
+          <t xml:space="preserve">brand</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
@@ -916,7 +945,7 @@
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">รุ่น เช่น SUN2000-100KTL</t>
+          <t xml:space="preserve">ยี่ห้อ เช่น Huawei, Growatt, Delta</t>
         </is>
       </c>
     </row>
@@ -928,7 +957,7 @@
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">serial_number</t>
+          <t xml:space="preserve">model</t>
         </is>
       </c>
       <c r="C19" s="4" t="inlineStr">
@@ -943,7 +972,7 @@
       </c>
       <c r="E19" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">S/N ของอุปกรณ์ — ใช้เฉพาะ asset_type = object (ไม่บังคับให้ไม่ซ้ำ เพราะคนละยี่ห้อ S/N ซ้ำกันได้)</t>
+          <t xml:space="preserve">รุ่น เช่น SUN2000-100KTL</t>
         </is>
       </c>
     </row>
@@ -955,7 +984,7 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">project_number</t>
+          <t xml:space="preserve">serial_number</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
@@ -970,7 +999,7 @@
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">เลขที่โครงการ — ใช้เฉพาะ asset_type = project</t>
+          <t xml:space="preserve">S/N ของอุปกรณ์ — ใช้เฉพาะ asset_type = object (ไม่บังคับให้ไม่ซ้ำ เพราะคนละยี่ห้อ S/N ซ้ำกันได้)</t>
         </is>
       </c>
     </row>
@@ -982,7 +1011,7 @@
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">group_name</t>
+          <t xml:space="preserve">project_number</t>
         </is>
       </c>
       <c r="C21" s="4" t="inlineStr">
@@ -997,7 +1026,7 @@
       </c>
       <c r="E21" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">ชื่อกลุ่ม Asset ภายในไซต์ เช่น “อาคาร A” — ถ้ายังไม่มีกลุ่มนี้ในไซต์ ระบบจะไม่ผูกให้</t>
+          <t xml:space="preserve">เลขที่โครงการ — ใช้เฉพาะ asset_type = project</t>
         </is>
       </c>
     </row>
@@ -1009,7 +1038,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">install_date</t>
+          <t xml:space="preserve">group_name</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
@@ -1019,12 +1048,12 @@
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">วันที่ YYYY-MM-DD</t>
+          <t xml:space="preserve">ข้อความ</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">วันที่ติดตั้ง</t>
+          <t xml:space="preserve">ชื่อกลุ่ม Asset ภายในไซต์ เช่น “อาคาร A” — ถ้ายังไม่มีกลุ่มนี้ในไซต์ ระบบจะไม่ผูกให้</t>
         </is>
       </c>
     </row>
@@ -1036,7 +1065,7 @@
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">warranty_start</t>
+          <t xml:space="preserve">install_date</t>
         </is>
       </c>
       <c r="C23" s="4" t="inlineStr">
@@ -1051,7 +1080,7 @@
       </c>
       <c r="E23" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">วันที่เริ่มประกัน (ถ้าเว้นว่างจะไม่คำนวณวันหมดประกันให้)</t>
+          <t xml:space="preserve">วันที่ติดตั้ง</t>
         </is>
       </c>
     </row>
@@ -1063,7 +1092,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">warranty_months</t>
+          <t xml:space="preserve">warranty_start</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
@@ -1073,12 +1102,12 @@
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">จำนวนเต็ม</t>
+          <t xml:space="preserve">วันที่ YYYY-MM-DD</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">อายุประกันเป็นเดือน เช่น 60 = 5 ปี — วันหมดประกันคำนวณจาก warranty_start + จำนวนเดือนนี้</t>
+          <t xml:space="preserve">วันที่เริ่มประกัน (ถ้าเว้นว่างจะไม่คำนวณวันหมดประกันให้)</t>
         </is>
       </c>
     </row>
@@ -1090,7 +1119,7 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">status</t>
+          <t xml:space="preserve">warranty_months</t>
         </is>
       </c>
       <c r="C25" s="4" t="inlineStr">
@@ -1100,12 +1129,12 @@
       </c>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">ตัวเลือก: operational / degraded / down / retired</t>
+          <t xml:space="preserve">จำนวนเต็ม</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">สถานะเครื่อง: operational = ใช้งานได้, degraded = พอใช้งานได้, down = ใช้งานไม่ได้, retired = ปลดระวาง · เว้นว่าง = operational</t>
+          <t xml:space="preserve">อายุประกันเป็นเดือน เช่น 60 = 5 ปี — วันหมดประกันคำนวณจาก warranty_start + จำนวนเดือนนี้</t>
         </is>
       </c>
     </row>
@@ -1117,20 +1146,47 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">status</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ตัวเลือก: operational / degraded / down / retired</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">สถานะเครื่อง: operational = ใช้งานได้, degraded = พอใช้งานได้, down = ใช้งานไม่ได้, retired = ปลดระวาง · เว้นว่าง = operational</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">notes</t>
         </is>
       </c>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">—</t>
         </is>
       </c>
-      <c r="D26" s="8" t="inlineStr">
+      <c r="D27" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">ข้อความ</t>
         </is>
       </c>
-      <c r="E26" s="8" t="inlineStr">
+      <c r="E27" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">หมายเหตุ</t>
         </is>

</xml_diff>